<commit_message>
Remove pointless '% del grupo' column from Palabras ABE sheet
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_run/resultados_Examen.xlsx
+++ b/test_run/resultados_Examen.xlsx
@@ -646,7 +646,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>3</col>
       <colOff>0</colOff>
       <row>2</row>
       <rowOff>0</rowOff>
@@ -1032,7 +1032,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 13:02</t>
+          <t>Generado: 05/05/2026 13:04</t>
         </is>
       </c>
     </row>
@@ -2170,12 +2170,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -2196,11 +2195,6 @@
           <t>Selecciones</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>% del grupo</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="22" t="inlineStr">
@@ -2211,9 +2205,6 @@
       <c r="B4" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="C4" s="6" t="n">
-        <v>100</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="23" t="inlineStr">
@@ -2224,9 +2215,6 @@
       <c r="B5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C5" s="4" t="n">
-        <v>50</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="22" t="inlineStr">
@@ -2237,9 +2225,6 @@
       <c r="B6" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="6" t="n">
-        <v>25</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="23" t="inlineStr">
@@ -2250,9 +2235,6 @@
       <c r="B7" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="4" t="n">
-        <v>25</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="22" t="inlineStr">
@@ -2263,9 +2245,6 @@
       <c r="B8" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="6" t="n">
-        <v>50</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="23" t="inlineStr">
@@ -2276,9 +2255,6 @@
       <c r="B9" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="4" t="n">
-        <v>50</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="22" t="inlineStr">
@@ -2289,9 +2265,6 @@
       <c r="B10" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="6" t="n">
-        <v>25</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="23" t="inlineStr">
@@ -2302,9 +2275,6 @@
       <c r="B11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="4" t="n">
-        <v>25</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="22" t="inlineStr">
@@ -2315,9 +2285,6 @@
       <c r="B12" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="6" t="n">
-        <v>25</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="23" t="inlineStr">
@@ -2328,9 +2295,6 @@
       <c r="B13" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C13" s="4" t="n">
-        <v>25</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="22" t="inlineStr">
@@ -2341,9 +2305,6 @@
       <c r="B14" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="C14" s="6" t="n">
-        <v>25</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="23" t="inlineStr">
@@ -2354,13 +2315,10 @@
       <c r="B15" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C15" s="4" t="n">
-        <v>25</v>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Improve Gráficas sheet: add Nombre column, styled data table, cleaner charts
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_run/resultados_Examen.xlsx
+++ b/test_run/resultados_Examen.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -92,12 +92,6 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="002C3E50"/>
-      <sz val="14"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -174,7 +168,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -237,14 +231,13 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -423,7 +416,7 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+  <style val="2"/>
   <chart>
     <title>
       <tx>
@@ -434,7 +427,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Puntaje por Estudiante (%)</a:t>
+              <a:t>Sección 1 — Puntaje de Opción Múltiple (%)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -449,22 +442,28 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Gráficas'!B3</f>
+              <f>'Gráficas'!E4</f>
             </strRef>
           </tx>
           <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="3498DB"/>
+            </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
+                <a:srgbClr val="3498DB"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Gráficas'!$A$4:$A$7</f>
+              <f>'Gráficas'!$B$5:$B$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Gráficas'!$B$4:$B$7</f>
+              <f>'Gráficas'!$E$5:$E$8</f>
             </numRef>
           </val>
         </ser>
@@ -487,7 +486,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Folio</a:t>
+                  <a:t>Estudiante</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -516,7 +515,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Porcentaje</a:t>
+                  <a:t>Porcentaje (%)</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -538,7 +537,7 @@
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+  <style val="2"/>
   <chart>
     <title>
       <tx>
@@ -549,7 +548,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Promedio Autoconocimiento</a:t>
+              <a:t>Sección 2 — Promedio de Autoconocimiento</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -563,11 +562,14 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Gráficas'!C3</f>
+              <f>'Gráficas'!F4</f>
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25000">
+              <a:solidFill>
+                <a:srgbClr val="E74C3C"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -581,12 +583,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Gráficas'!$A$4:$A$7</f>
+              <f>'Gráficas'!$B$5:$B$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Gráficas'!$C$4:$C$7</f>
+              <f>'Gráficas'!$F$5:$F$8</f>
             </numRef>
           </val>
         </ser>
@@ -599,6 +601,21 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Estudiante</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -622,7 +639,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Promedio (1-5)</a:t>
+                  <a:t>Promedio (1–5)</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -673,12 +690,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>8</col>
       <colOff>0</colOff>
-      <row>2</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7200000" cy="4320000"/>
+    <ext cx="8640000" cy="5040000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -695,12 +712,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>8</col>
       <colOff>0</colOff>
-      <row>22</row>
+      <row>26</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7200000" cy="4320000"/>
+    <ext cx="8640000" cy="5040000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -1032,7 +1049,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 13:04</t>
+          <t>Generado: 05/05/2026 13:08</t>
         </is>
       </c>
     </row>
@@ -2331,143 +2348,180 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="24" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Gráficas de Resultados</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Generado: 05/05/2026 13:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Folio</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Porcentaje</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Prom. SK</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Grado</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>Grupo</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
+        <is>
+          <t>Puntaje MC (%)</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Prom. Autoconoc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Ana García López</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="C4" t="n">
+      <c r="F5" s="4" t="n">
         <v>3.9</v>
       </c>
-      <c r="D4" t="inlineStr">
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Carlos Mendoza Ruiz</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n">
         <v>90</v>
       </c>
-      <c r="C5" t="n">
+      <c r="F6" s="6" t="n">
         <v>3.4</v>
       </c>
-      <c r="D5" t="inlineStr">
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Sofia Torres Vega</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>47</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n">
         <v>90</v>
       </c>
-      <c r="C6" t="n">
+      <c r="F7" s="4" t="n">
         <v>4.7</v>
       </c>
-      <c r="D6" t="inlineStr">
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Roberto Jiménez Cruz</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>63</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="n">
         <v>90</v>
       </c>
-      <c r="C7" t="n">
+      <c r="F8" s="6" t="n">
         <v>2.6</v>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -2503,94 +2557,94 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="25" t="inlineStr">
+      <c r="A3" s="24" t="inlineStr">
         <is>
           <t>Pregunta</t>
         </is>
       </c>
-      <c r="B3" s="25" t="n">
+      <c r="B3" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="25" t="n">
+      <c r="C3" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="25" t="n">
+      <c r="D3" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="E3" s="25" t="n">
+      <c r="E3" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="F3" s="25" t="n">
+      <c r="F3" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="G3" s="25" t="n">
+      <c r="G3" s="24" t="n">
         <v>6</v>
       </c>
-      <c r="H3" s="25" t="n">
+      <c r="H3" s="24" t="n">
         <v>7</v>
       </c>
-      <c r="I3" s="25" t="n">
+      <c r="I3" s="24" t="n">
         <v>8</v>
       </c>
-      <c r="J3" s="25" t="n">
+      <c r="J3" s="24" t="n">
         <v>9</v>
       </c>
-      <c r="K3" s="25" t="n">
+      <c r="K3" s="24" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="26" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>Respuesta</t>
         </is>
       </c>
-      <c r="B4" s="27" t="inlineStr">
+      <c r="B4" s="26" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C4" s="27" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D4" s="27" t="inlineStr">
+      <c r="C4" s="26" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D4" s="26" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="E4" s="27" t="inlineStr">
+      <c r="E4" s="26" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="F4" s="27" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G4" s="27" t="inlineStr">
+      <c r="F4" s="26" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G4" s="26" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H4" s="27" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="I4" s="27" t="inlineStr">
+      <c r="H4" s="26" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I4" s="26" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="J4" s="27" t="inlineStr">
+      <c r="J4" s="26" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="K4" s="27" t="inlineStr">
+      <c r="K4" s="26" t="inlineStr">
         <is>
           <t>A</t>
         </is>

</xml_diff>

<commit_message>
Group charts by Grado+Grupo instead of individual students
Gráficas sheet now shows a group summary table with averages per
Grado/Grupo combination, and both charts (MC % and Autoconocimiento)
plot those group averages so results across grades are comparable.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_run/resultados_Examen.xlsx
+++ b/test_run/resultados_Examen.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -92,6 +92,12 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -168,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -231,13 +237,16 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -427,7 +436,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Sección 1 — Puntaje de Opción Múltiple (%)</a:t>
+              <a:t>Sección 1 — Puntaje Promedio por Grupo (%)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -442,7 +451,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Gráficas'!E4</f>
+              <f>'Gráficas'!C11</f>
             </strRef>
           </tx>
           <spPr>
@@ -458,12 +467,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Gráficas'!$B$5:$B$8</f>
+              <f>'Gráficas'!$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Gráficas'!$E$5:$E$8</f>
+              <f>'Gráficas'!$C$12</f>
             </numRef>
           </val>
         </ser>
@@ -486,7 +495,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Estudiante</a:t>
+                  <a:t>Grupo</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -548,53 +557,50 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Sección 2 — Promedio de Autoconocimiento</a:t>
+              <a:t>Sección 2 — Promedio de Autoconocimiento por Grupo</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
     </title>
     <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Gráficas'!F4</f>
+              <f>'Gráficas'!D11</f>
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25000">
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="E74C3C"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="E74C3C"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
           <cat>
             <numRef>
-              <f>'Gráficas'!$B$5:$B$8</f>
+              <f>'Gráficas'!$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Gráficas'!$F$5:$F$8</f>
+              <f>'Gráficas'!$D$12</f>
             </numRef>
           </val>
         </ser>
+        <gapWidth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
-      </lineChart>
+      </barChart>
       <catAx>
         <axId val="10"/>
         <scaling>
@@ -610,7 +616,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Estudiante</a:t>
+                  <a:t>Grupo</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -690,12 +696,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>8</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8640000" cy="5040000"/>
+    <ext cx="7920000" cy="5040000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -712,12 +718,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>8</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>26</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8640000" cy="5040000"/>
+    <ext cx="7920000" cy="5040000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -1049,7 +1055,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 13:08</t>
+          <t>Generado: 05/05/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -2348,13 +2354,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
@@ -2369,7 +2375,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 13:08</t>
+          <t>Generado: 05/05/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -2517,8 +2523,54 @@
         <v>2.6</v>
       </c>
     </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>Resumen por Grado y Grupo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Grado / Grupo</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>N Alumnos</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>Prom. MC (%)</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>Prom. Autoconoc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="22" t="inlineStr">
+        <is>
+          <t>Grado 2 / Grupo B</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>92.5</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A10:D10"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
@@ -2557,94 +2609,94 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="24" t="inlineStr">
+      <c r="A3" s="25" t="inlineStr">
         <is>
           <t>Pregunta</t>
         </is>
       </c>
-      <c r="B3" s="24" t="n">
+      <c r="B3" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="24" t="n">
+      <c r="C3" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="24" t="n">
+      <c r="D3" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="E3" s="24" t="n">
+      <c r="E3" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="F3" s="24" t="n">
+      <c r="F3" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="G3" s="24" t="n">
+      <c r="G3" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="H3" s="24" t="n">
+      <c r="H3" s="25" t="n">
         <v>7</v>
       </c>
-      <c r="I3" s="24" t="n">
+      <c r="I3" s="25" t="n">
         <v>8</v>
       </c>
-      <c r="J3" s="24" t="n">
+      <c r="J3" s="25" t="n">
         <v>9</v>
       </c>
-      <c r="K3" s="24" t="n">
+      <c r="K3" s="25" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="25" t="inlineStr">
+      <c r="A4" s="26" t="inlineStr">
         <is>
           <t>Respuesta</t>
         </is>
       </c>
-      <c r="B4" s="26" t="inlineStr">
+      <c r="B4" s="27" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C4" s="26" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D4" s="26" t="inlineStr">
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="E4" s="26" t="inlineStr">
+      <c r="E4" s="27" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="F4" s="26" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G4" s="26" t="inlineStr">
+      <c r="F4" s="27" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G4" s="27" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H4" s="26" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="I4" s="26" t="inlineStr">
+      <c r="H4" s="27" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I4" s="27" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="J4" s="26" t="inlineStr">
+      <c r="J4" s="27" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="K4" s="26" t="inlineStr">
+      <c r="K4" s="27" t="inlineStr">
         <is>
           <t>A</t>
         </is>

</xml_diff>